<commit_message>
feat(masterdata): MountedArchery 체력·화살 위력·되감기 상한
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#MountedArcheryConfig.xlsx
+++ b/table/Datas/#MountedArcheryConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,6 +487,21 @@
           <t>draw_speed_factor</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>max_hp</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>arrow_damage</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>lag_comp_max_seconds</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -559,6 +574,21 @@
           <t>float</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -636,6 +666,21 @@
       <c r="N4" t="inlineStr">
         <is>
           <t>draw_speed_factor</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>max_hp</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>arrow_damage</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>lag_comp_max_seconds</t>
         </is>
       </c>
     </row>
@@ -677,6 +722,15 @@
         <v>0.35</v>
       </c>
       <c r="N5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O5" t="n">
+        <v>100</v>
+      </c>
+      <c r="P5" t="n">
+        <v>34</v>
+      </c>
+      <c r="Q5" t="n">
         <v>0.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(masterdata): MountedArchery 원 단계 표와 조준 보정 수치
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#MountedArcheryConfig.xlsx
+++ b/table/Datas/#MountedArcheryConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,6 +502,36 @@
           <t>lag_comp_max_seconds</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>zone_initial_radius</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>zone_first_reveal_seconds</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>aim_assist_cone_deg</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>aim_assist_range</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>aim_assist_friction</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>aim_assist_track</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -589,6 +619,36 @@
           <t>float</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -681,6 +741,36 @@
       <c r="Q4" t="inlineStr">
         <is>
           <t>lag_comp_max_seconds</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>zone_initial_radius</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>zone_first_reveal_seconds</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>aim_assist_cone_deg</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>aim_assist_range</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>aim_assist_friction</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>aim_assist_track</t>
         </is>
       </c>
     </row>
@@ -731,6 +821,24 @@
         <v>34</v>
       </c>
       <c r="Q5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="R5" t="n">
+        <v>100</v>
+      </c>
+      <c r="S5" t="n">
+        <v>30</v>
+      </c>
+      <c r="T5" t="n">
+        <v>4</v>
+      </c>
+      <c r="U5" t="n">
+        <v>90</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="W5" t="n">
         <v>0.5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(masterdata): MountedArchery 판 길이 180초와 마지막 원 뒤 피해 증가량
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#MountedArcheryConfig.xlsx
+++ b/table/Datas/#MountedArcheryConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W5"/>
+  <dimension ref="A1:X5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -532,6 +532,11 @@
           <t>aim_assist_track</t>
         </is>
       </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>zone_overtime_dps_growth</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -649,6 +654,11 @@
           <t>float</t>
         </is>
       </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -771,6 +781,11 @@
       <c r="W4" t="inlineStr">
         <is>
           <t>aim_assist_track</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>zone_overtime_dps_growth</t>
         </is>
       </c>
     </row>
@@ -779,7 +794,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="D5" t="n">
         <v>26</v>
@@ -840,6 +855,9 @@
       </c>
       <c r="W5" t="n">
         <v>0.5</v>
+      </c>
+      <c r="X5" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(masterdata): MountedArchery 후진 최고 속도 mount_reverse_speed 3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#MountedArcheryConfig.xlsx
+++ b/table/Datas/#MountedArcheryConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X5"/>
+  <dimension ref="A1:Y5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,6 +537,11 @@
           <t>zone_overtime_dps_growth</t>
         </is>
       </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>mount_reverse_speed</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -659,6 +664,11 @@
           <t>float</t>
         </is>
       </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -786,6 +796,11 @@
       <c r="X4" t="inlineStr">
         <is>
           <t>zone_overtime_dps_growth</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>mount_reverse_speed</t>
         </is>
       </c>
     </row>
@@ -858,6 +873,9 @@
       </c>
       <c r="X5" t="n">
         <v>15</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(masterdata): MountedArchery 만작 시간 full_draw_seconds 0.35
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#MountedArcheryConfig.xlsx
+++ b/table/Datas/#MountedArcheryConfig.xlsx
@@ -413,8 +413,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC5"/>
+  <dimension ref="A1:AD5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -562,6 +566,11 @@
           <t>bot_engage_range</t>
         </is>
       </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>full_draw_seconds</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -709,6 +718,11 @@
           <t>float</t>
         </is>
       </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -861,6 +875,11 @@
       <c r="AC4" t="inlineStr">
         <is>
           <t>bot_engage_range</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>full_draw_seconds</t>
         </is>
       </c>
     </row>
@@ -948,6 +967,9 @@
       </c>
       <c r="AC5" t="n">
         <v>60</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tune(mounted-archery): 말 최고 속도 13→7, 당기는 동안 속도 배율 0.5→0.2
실플레이(폰): 말이 너무 빨라 겨누기 어렵다 — 달릴 땐 이동, 겨눌 땐 거의 서서 정확하게를 시험한다.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#MountedArcheryConfig.xlsx
+++ b/table/Datas/#MountedArcheryConfig.xlsx
@@ -900,7 +900,7 @@
         <v>2.5</v>
       </c>
       <c r="G5" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="H5" t="n">
         <v>9</v>
@@ -921,7 +921,7 @@
         <v>0.35</v>
       </c>
       <c r="N5" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="O5" t="n">
         <v>100</v>

</xml_diff>